<commit_message>
Updated workbook with temperature trend analysis
</commit_message>
<xml_diff>
--- a/pakistan_temperature_analysis.xlsx
+++ b/pakistan_temperature_analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uk094843\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0FC3BFB-7A53-4C38-A151-B56DA25A73A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8AF17B-5884-40A8-BD2D-C12CE8350CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="137">
   <si>
     <t>code</t>
   </si>
@@ -453,6 +453,12 @@
   </si>
   <si>
     <t>Difference</t>
+  </si>
+  <si>
+    <t>Estimated temperature trend (°C/year)</t>
+  </si>
+  <si>
+    <t>Estimated temperature trend (°C/decade)</t>
   </si>
 </sst>
 </file>
@@ -562,7 +568,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -575,10 +581,10 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
               <a:t>Pakistan: Annual Average Surface Air Temperature, 1901–2025</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="en-US" sz="1200"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -595,7 +601,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -613,7 +619,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.12537314220956097"/>
+          <c:y val="0.19104143337066071"/>
+          <c:w val="0.82926195922625912"/>
+          <c:h val="0.58303127562582113"/>
+        </c:manualLayout>
+      </c:layout>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -2262,16 +2278,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>498474</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>174624</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>53975</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>53975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>177798</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>12699</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>57148</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2866,6 +2882,13 @@
       <c r="E5">
         <v>1904</v>
       </c>
+      <c r="G5" t="s">
+        <v>135</v>
+      </c>
+      <c r="H5">
+        <f>SLOPE(D2:D126,E2:E126)</f>
+        <v>9.4345929339477736E-3</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.75">
       <c r="A6" s="2" t="s">
@@ -2882,6 +2905,13 @@
       </c>
       <c r="E6">
         <v>1905</v>
+      </c>
+      <c r="G6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H6">
+        <f>H5*10</f>
+        <v>9.4345929339477733E-2</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.75">

</xml_diff>